<commit_message>
PAUSED (task140): write-up figures at the precision every variant shares, re-read next
Precision-only change to blocks 1 and 2, accepted by the main session:
Critical Component 4 is the 1.208 reservable cores each guaranteed core
takes (109,492 dropped), Component 3 has no parentheses, the Final
Recommendation's coefficients read 2.94 and 0.208. Block 3 and the goldens
follow (the 2027 Q1 sheet's platform rows at the thousand, the cell-store
sheet's terms at 2.94 and 0.208, the slide's remainder as under 1,000). No
graded figure, file under target/ or figures.json value moved (three keys
added); checks.py asserts the shared precision under every converging
variant. freeze.py snapshot retaken after the change. The main session's
targeted re-read kept in leak_check_report.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task140/golden/c22_capacity_2027q1.xlsx
+++ b/task140/golden/c22_capacity_2027q1.xlsx
@@ -72,7 +72,7 @@
     <t>cell-store</t>
   </si>
   <si>
-    <t>Busiest hour forecast from its drivers: 33.1 + 2.9404 per machine in service + 0.20804 per batch core running, at 5,220 machines and batch at its guarantee (sheet cell-store)</t>
+    <t>Busiest hour forecast from its drivers: 2.94 cores per machine in service and 0.208 per batch core running, at 5,220 machines and batch at its guarantee (sheet cell-store)</t>
   </si>
   <si>
     <t>Platform services</t>
@@ -84,16 +84,16 @@
     <t>Batch training guarantee</t>
   </si>
   <si>
-    <t>Largest whole thousand left; solved with cell-store, which rises by 0.20804 cores for each batch core: (726,624 - firm - cell-ctl - 33.1 - 2.9404 x 5,220) / 1.20804 = 109,492.0</t>
+    <t>Largest whole thousand left, solved together with cell-store: each guaranteed core takes 1.208 reservable cores, its own and 0.208 of cell-store load</t>
   </si>
   <si>
     <t>Not reserved</t>
   </si>
   <si>
-    <t>Left after the guarantee (CS-3 5.2)</t>
-  </si>
-  <si>
-    <t>For comparison: carrying cell-store forward on its own last four busiest hours (25,418 cores) would leave 122,000 cores, but every batch core added brings 0.20804 cores of cell-store load that history at a guarantee of 55,000 to 58,000 cores has not seen.</t>
+    <t>Left after the guarantee, under 1,000 cores (CS-3 5.2)</t>
+  </si>
+  <si>
+    <t>For comparison: carrying cell-store forward on its own last four busiest hours (25,418 cores) would leave 122,000 cores, but every batch core added brings 0.208 cores of cell-store load that history at a guarantee of 55,000 to 58,000 cores has not seen.</t>
   </si>
   <si>
     <t>Firm tenants: Q1 2027 requests held to frozen budgets</t>
@@ -282,7 +282,7 @@
     <t>2026-12-10 18:00</t>
   </si>
   <si>
-    <t>2027 Q1 at 5,220 machines, batch at 109,000</t>
+    <t>2027 Q1 at 5,220 machines, batch at 109,000 (reserved, nearest 1,000)</t>
   </si>
   <si>
     <t>Batch training lost to preemptions, July to September 2026</t>
@@ -403,11 +403,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
-    <numFmt numFmtId="167" formatCode="0.00000"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -483,7 +482,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -505,10 +504,8 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -890,9 +887,7 @@
       <c r="A8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="7">
-        <v>1999.2</v>
-      </c>
+      <c r="B8" s="7"/>
       <c r="C8" s="5">
         <v>2000</v>
       </c>
@@ -904,9 +899,7 @@
       <c r="A9" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="7">
-        <v>38058.5</v>
-      </c>
+      <c r="B9" s="7"/>
       <c r="C9" s="5">
         <v>38000</v>
       </c>
@@ -918,9 +911,7 @@
       <c r="A10" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="7">
-        <v>40057.7</v>
-      </c>
+      <c r="B10" s="7"/>
       <c r="C10" s="5">
         <v>40000</v>
       </c>
@@ -946,11 +937,9 @@
       <c r="A12" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="7">
-        <v>594.3</v>
-      </c>
+      <c r="B12" s="7"/>
       <c r="C12" s="5"/>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="4" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1339,7 +1328,7 @@
         <v>61</v>
       </c>
       <c r="B6" s="13">
-        <v>2.9404</v>
+        <v>2.94</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1347,7 +1336,7 @@
         <v>62</v>
       </c>
       <c r="B7" s="14">
-        <v>0.20804</v>
+        <v>0.208</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1387,7 +1376,7 @@
         <v>55974.1</v>
       </c>
       <c r="F10" s="7">
-        <v>24198.2</v>
+        <v>24194.2</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1407,7 +1396,7 @@
         <v>57979.3</v>
       </c>
       <c r="F11" s="7">
-        <v>24738.9</v>
+        <v>24734.8</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1427,7 +1416,7 @@
         <v>54969.1</v>
       </c>
       <c r="F12" s="7">
-        <v>24286.1</v>
+        <v>24282.1</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1447,7 +1436,7 @@
         <v>56996</v>
       </c>
       <c r="F13" s="7">
-        <v>24822.4</v>
+        <v>24818.4</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1467,7 +1456,7 @@
         <v>57983.4</v>
       </c>
       <c r="F14" s="7">
-        <v>25200.8</v>
+        <v>25196.6</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1487,7 +1476,7 @@
         <v>54995.2</v>
       </c>
       <c r="F15" s="7">
-        <v>24759</v>
+        <v>24755</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1507,7 +1496,7 @@
         <v>56817.5</v>
       </c>
       <c r="F16" s="7">
-        <v>25320.5</v>
+        <v>25316.3</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1527,7 +1516,7 @@
         <v>55991.7</v>
       </c>
       <c r="F17" s="7">
-        <v>25318.6</v>
+        <v>25314.5</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1535,8 +1524,8 @@
         <v>85</v>
       </c>
       <c r="B19" s="8"/>
-      <c r="C19" s="15">
-        <v>38058.5</v>
+      <c r="C19" s="9">
+        <v>38000</v>
       </c>
     </row>
   </sheetData>
@@ -1593,7 +1582,7 @@
       <c r="C5" s="5">
         <v>121800</v>
       </c>
-      <c r="D5" s="16">
+      <c r="D5" s="13">
         <v>0.4</v>
       </c>
     </row>
@@ -1607,7 +1596,7 @@
       <c r="C6" s="5">
         <v>80500</v>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="13">
         <v>0.37</v>
       </c>
     </row>
@@ -1621,7 +1610,7 @@
       <c r="C7" s="5">
         <v>48500</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="13">
         <v>0.31</v>
       </c>
     </row>
@@ -1635,7 +1624,7 @@
       <c r="C8" s="5">
         <v>144300</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="13">
         <v>0.59</v>
       </c>
     </row>
@@ -1649,7 +1638,7 @@
       <c r="C9" s="5">
         <v>72000</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="13">
         <v>0.49</v>
       </c>
     </row>
@@ -1663,7 +1652,7 @@
       <c r="C10" s="5">
         <v>134900</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="13">
         <v>0.77</v>
       </c>
     </row>
@@ -1752,7 +1741,7 @@
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="15" t="s">
         <v>106</v>
       </c>
     </row>
@@ -1927,7 +1916,7 @@
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="15" t="s">
         <v>111</v>
       </c>
     </row>

</xml_diff>

<commit_message>
PAUSED (task140): realism repair, stage 4 next
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task140/golden/c22_capacity_2027q1.xlsx
+++ b/task140/golden/c22_capacity_2027q1.xlsx
@@ -93,7 +93,7 @@
     <t>Left after the guarantee, under 1,000 cores (CS-3 5.2)</t>
   </si>
   <si>
-    <t>For comparison: carrying cell-store forward on its own last four busiest hours (25,418 cores) would leave 122,000 cores, but every batch core added brings 0.208 cores of cell-store load that history at a guarantee of 55,000 to 58,000 cores has not seen.</t>
+    <t>For comparison: carrying cell-store forward on its own last four busiest hours (25,486 cores) would leave 122,000 cores, but every batch core added brings 0.208 cores of cell-store load that history at a guarantee of 55,000 to 58,000 cores has not seen.</t>
   </si>
   <si>
     <t>Firm tenants: Q1 2027 requests held to frozen budgets</t>
@@ -201,7 +201,7 @@
     <t>cell-store: busiest-hour forecast from its drivers</t>
   </si>
   <si>
-    <t>Least squares on every hour on file (17,081 hours, 2025-01-01 to 2026-12-13): cell-store's cores in use on the cell's machines in service and the batch tier's cores in use. Residual s.d. 13.0 cores.</t>
+    <t>Least squares on every hour on file (17,081 hours, 2025-01-01 to 2026-12-13): cell-store's cores in use on the cell's machines in service and the batch tier's cores in use. Residual s.d. 62.0 cores; the low residuals are the Tuesday restart hours and hours whose samples reached the collector late.</t>
   </si>
   <si>
     <t>Term</t>
@@ -237,37 +237,37 @@
     <t>2025Q1</t>
   </si>
   <si>
-    <t>2025-03-27 14:00</t>
+    <t>2025-03-25 20:00</t>
   </si>
   <si>
     <t>2025Q2</t>
   </si>
   <si>
-    <t>2025-05-27 11:00</t>
+    <t>2025-06-01 21:00</t>
   </si>
   <si>
     <t>2025Q3</t>
   </si>
   <si>
-    <t>2025-09-19 04:00</t>
+    <t>2025-09-23 23:00</t>
   </si>
   <si>
     <t>2025Q4</t>
   </si>
   <si>
-    <t>2025-12-26 20:00</t>
+    <t>2025-11-30 11:00</t>
   </si>
   <si>
     <t>2026Q1</t>
   </si>
   <si>
-    <t>2026-03-24 23:00</t>
+    <t>2026-03-12 19:00</t>
   </si>
   <si>
     <t>2026Q2</t>
   </si>
   <si>
-    <t>2026-06-25 21:00</t>
+    <t>2026-06-29 11:00</t>
   </si>
   <si>
     <t>2026Q3</t>
@@ -1320,7 +1320,7 @@
         <v>60</v>
       </c>
       <c r="B5" s="12">
-        <v>33.1</v>
+        <v>39.1</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1367,16 +1367,16 @@
         <v>70</v>
       </c>
       <c r="C10" s="7">
-        <v>24233.3</v>
+        <v>24270.6</v>
       </c>
       <c r="D10" s="7">
-        <v>4258</v>
+        <v>4259</v>
       </c>
       <c r="E10" s="7">
-        <v>55974.1</v>
+        <v>55958.9</v>
       </c>
       <c r="F10" s="7">
-        <v>24194.2</v>
+        <v>24200</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1387,16 +1387,16 @@
         <v>72</v>
       </c>
       <c r="C11" s="7">
-        <v>24767.7</v>
+        <v>24805.3</v>
       </c>
       <c r="D11" s="7">
-        <v>4300</v>
+        <v>4299</v>
       </c>
       <c r="E11" s="7">
-        <v>57979.3</v>
+        <v>57978</v>
       </c>
       <c r="F11" s="7">
-        <v>24734.8</v>
+        <v>24737.6</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1407,16 +1407,16 @@
         <v>74</v>
       </c>
       <c r="C12" s="7">
-        <v>24320.1</v>
+        <v>24356.3</v>
       </c>
       <c r="D12" s="7">
-        <v>4359</v>
+        <v>4357</v>
       </c>
       <c r="E12" s="7">
-        <v>54969.1</v>
+        <v>54938</v>
       </c>
       <c r="F12" s="7">
-        <v>24282.1</v>
+        <v>24275.8</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1427,16 +1427,16 @@
         <v>76</v>
       </c>
       <c r="C13" s="7">
-        <v>24843.1</v>
+        <v>24879.7</v>
       </c>
       <c r="D13" s="7">
-        <v>4398</v>
+        <v>4397.3</v>
       </c>
       <c r="E13" s="7">
-        <v>56996</v>
+        <v>56929.4</v>
       </c>
       <c r="F13" s="7">
-        <v>24818.4</v>
+        <v>24808.5</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1447,16 +1447,16 @@
         <v>78</v>
       </c>
       <c r="C14" s="7">
-        <v>25233.1</v>
+        <v>25263.2</v>
       </c>
       <c r="D14" s="7">
-        <v>4456.8</v>
+        <v>4454.5</v>
       </c>
       <c r="E14" s="7">
-        <v>57983.4</v>
+        <v>57992.7</v>
       </c>
       <c r="F14" s="7">
-        <v>25196.6</v>
+        <v>25197.8</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1467,16 +1467,16 @@
         <v>80</v>
       </c>
       <c r="C15" s="7">
-        <v>24782.2</v>
+        <v>24816.7</v>
       </c>
       <c r="D15" s="7">
         <v>4518</v>
       </c>
       <c r="E15" s="7">
-        <v>54995.2</v>
+        <v>54941.1</v>
       </c>
       <c r="F15" s="7">
-        <v>24755</v>
+        <v>24749.8</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1487,7 +1487,7 @@
         <v>82</v>
       </c>
       <c r="C16" s="7">
-        <v>25359.1</v>
+        <v>25415.5</v>
       </c>
       <c r="D16" s="7">
         <v>4580</v>
@@ -1496,7 +1496,7 @@
         <v>56817.5</v>
       </c>
       <c r="F16" s="7">
-        <v>25316.3</v>
+        <v>25322.3</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1507,7 +1507,7 @@
         <v>84</v>
       </c>
       <c r="C17" s="7">
-        <v>25354.6</v>
+        <v>25410</v>
       </c>
       <c r="D17" s="7">
         <v>4637.8</v>
@@ -1516,7 +1516,7 @@
         <v>55991.7</v>
       </c>
       <c r="F17" s="7">
-        <v>25314.5</v>
+        <v>25320.5</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>